<commit_message>
메일 추가 요청(2) — Cummins 분석 시트 Promise Date → 대장 EXW DATE (Undispatched·HCE, 분할 선적 수량 대조, 노란 줄 확인)
- 새 화면 「Cummins EXW」: 분석 시트 자동 선택, Status·구분 거르기(기본 Undispatched·HCE), PO+Part No. 로 대장과 맞춤
- 날짜별 수량(분할 선적), 파일 수량 합 vs PO(초기 발주)·OC 수량 부족·초과 표시, 일치 건만 미리 선택·불일치는 확인 후 반영
- 노란 채우기(SheetJS cellStyles) → 변경 확인 필요, 색 없이도 EXW 바뀜 판정, 반영 전/후 표·엑셀, 대장에 없음/파일에 없음
- 대장에 품번별 출하 일정(exw_plan)·OC 품목 수량(oc_lines) 저장
- 가상 예시(노란 줄·분할·불일치 포함 xlsx), 시험 79 → 87개, 기획서 11.5

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/예시데이터_관리대장.xlsx
+++ b/samples/예시데이터_관리대장.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R11"/>
+  <dimension ref="A1:S11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -452,6 +452,9 @@
         <v>OC 번호</v>
       </c>
       <c r="R1" t="str">
+        <v>EXW 일정(품번별)</v>
+      </c>
+      <c r="S1" t="str">
         <v>항차 진행</v>
       </c>
     </row>
@@ -508,6 +511,9 @@
         <v/>
       </c>
       <c r="R2" t="str">
+        <v/>
+      </c>
+      <c r="S2" t="str">
         <v>4/13</v>
       </c>
     </row>
@@ -564,6 +570,9 @@
         <v/>
       </c>
       <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
         <v>4/13</v>
       </c>
     </row>
@@ -620,6 +629,9 @@
         <v/>
       </c>
       <c r="R4" t="str">
+        <v/>
+      </c>
+      <c r="S4" t="str">
         <v>4/13</v>
       </c>
     </row>
@@ -676,6 +688,9 @@
         <v/>
       </c>
       <c r="R5" t="str">
+        <v/>
+      </c>
+      <c r="S5" t="str">
         <v>3/13</v>
       </c>
     </row>
@@ -732,6 +747,9 @@
         <v/>
       </c>
       <c r="R6" t="str">
+        <v/>
+      </c>
+      <c r="S6" t="str">
         <v>3/13</v>
       </c>
     </row>
@@ -788,6 +806,9 @@
         <v/>
       </c>
       <c r="R7" t="str">
+        <v/>
+      </c>
+      <c r="S7" t="str">
         <v>1/13</v>
       </c>
     </row>
@@ -844,6 +865,9 @@
         <v/>
       </c>
       <c r="R8" t="str">
+        <v/>
+      </c>
+      <c r="S8" t="str">
         <v>1/13</v>
       </c>
     </row>
@@ -900,6 +924,9 @@
         <v/>
       </c>
       <c r="R9" t="str">
+        <v/>
+      </c>
+      <c r="S9" t="str">
         <v>1/13</v>
       </c>
     </row>
@@ -956,6 +983,9 @@
         <v/>
       </c>
       <c r="R10" t="str">
+        <v/>
+      </c>
+      <c r="S10" t="str">
         <v>3/13</v>
       </c>
     </row>
@@ -1012,12 +1042,15 @@
         <v/>
       </c>
       <c r="R11" t="str">
+        <v/>
+      </c>
+      <c r="S11" t="str">
         <v>1/13</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>